<commit_message>
Various improvements and fixes (#74)
- Added option to adjust the fixed loop time. Removed the hard-coded value.
- Redesigned the system menu. Disbanded the Advanced sub-menu, moved the About sub-menu to the main menu.
- Improved the timings for failsafe, telemetry, and when binding. Significantly reduced the delay between switching on the receiver and getting the very first signal on the output pin. This fixes an issue where certain ESCs sometimes fail to respond to the throttle signal.
- The SPI clock frequency can now be specified in the config.h files. This fixes an issue with some level shifters not supporting very high speeds.
- Other minor improvements.
</commit_message>
<xml_diff>
--- a/doc/spreadsheets/timing_failsafe_telemetry.xlsx
+++ b/doc/spreadsheets/timing_failsafe_telemetry.xlsx
@@ -1,23 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ba\rc radio project\New stuff\Beta36\doc\spreadsheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ba\rc radio project\New stuff\Beta43\doc\spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C6E939-3C5E-40D6-B19E-5DED827DE32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7224"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="10416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -35,13 +47,13 @@
     <t>Time (ms)</t>
   </si>
   <si>
-    <t>Modulo 64</t>
+    <t>Modulo 32</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -359,7 +371,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F9254A-C71B-4C3E-94C8-9BE104737D94}">
   <dimension ref="A2:D504"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -391,11 +403,11 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <f>MOD(A5,64)</f>
+        <f>MOD(A5,32)</f>
         <v>1</v>
       </c>
       <c r="C5" t="str">
-        <f>IF(B5=16, "Failsafe",IF(OR(B5=0,B5=32),"telemetry",""))</f>
+        <f>IF(B5=16, "Failsafe",IF(B5=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D5">
@@ -408,11 +420,11 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <f t="shared" ref="B6:B69" si="0">MOD(A6,64)</f>
+        <f t="shared" ref="B6:B69" si="0">MOD(A6,32)</f>
         <v>2</v>
       </c>
       <c r="C6" t="str">
-        <f t="shared" ref="C6:C69" si="1">IF(B6=16, "Failsafe",IF(OR(B6=0,B6=32),"telemetry",""))</f>
+        <f t="shared" ref="C6:C69" si="1">IF(B6=16, "Failsafe",IF(B6=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D6">
@@ -919,7 +931,7 @@
       </c>
       <c r="B36">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="1"/>
@@ -936,7 +948,7 @@
       </c>
       <c r="B37">
         <f t="shared" si="0"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="1"/>
@@ -953,7 +965,7 @@
       </c>
       <c r="B38">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="1"/>
@@ -970,7 +982,7 @@
       </c>
       <c r="B39">
         <f t="shared" si="0"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C39" t="str">
         <f t="shared" si="1"/>
@@ -987,7 +999,7 @@
       </c>
       <c r="B40">
         <f t="shared" si="0"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="1"/>
@@ -1004,7 +1016,7 @@
       </c>
       <c r="B41">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="1"/>
@@ -1021,7 +1033,7 @@
       </c>
       <c r="B42">
         <f t="shared" si="0"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="1"/>
@@ -1038,7 +1050,7 @@
       </c>
       <c r="B43">
         <f t="shared" si="0"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C43" t="str">
         <f t="shared" si="1"/>
@@ -1055,7 +1067,7 @@
       </c>
       <c r="B44">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C44" t="str">
         <f t="shared" si="1"/>
@@ -1072,7 +1084,7 @@
       </c>
       <c r="B45">
         <f t="shared" si="0"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C45" t="str">
         <f t="shared" si="1"/>
@@ -1089,7 +1101,7 @@
       </c>
       <c r="B46">
         <f t="shared" si="0"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="1"/>
@@ -1106,7 +1118,7 @@
       </c>
       <c r="B47">
         <f t="shared" si="0"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="1"/>
@@ -1123,7 +1135,7 @@
       </c>
       <c r="B48">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="1"/>
@@ -1140,7 +1152,7 @@
       </c>
       <c r="B49">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C49" t="str">
         <f t="shared" si="1"/>
@@ -1157,7 +1169,7 @@
       </c>
       <c r="B50">
         <f t="shared" si="0"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C50" t="str">
         <f t="shared" si="1"/>
@@ -1174,7 +1186,7 @@
       </c>
       <c r="B51">
         <f t="shared" si="0"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C51" t="str">
         <f t="shared" si="1"/>
@@ -1191,11 +1203,11 @@
       </c>
       <c r="B52">
         <f t="shared" si="0"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C52" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D52">
         <f t="shared" si="2"/>
@@ -1208,7 +1220,7 @@
       </c>
       <c r="B53">
         <f t="shared" si="0"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C53" t="str">
         <f t="shared" si="1"/>
@@ -1225,7 +1237,7 @@
       </c>
       <c r="B54">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="1"/>
@@ -1242,7 +1254,7 @@
       </c>
       <c r="B55">
         <f t="shared" si="0"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="1"/>
@@ -1259,7 +1271,7 @@
       </c>
       <c r="B56">
         <f t="shared" si="0"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="1"/>
@@ -1276,7 +1288,7 @@
       </c>
       <c r="B57">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="1"/>
@@ -1293,7 +1305,7 @@
       </c>
       <c r="B58">
         <f t="shared" si="0"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="1"/>
@@ -1310,7 +1322,7 @@
       </c>
       <c r="B59">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="1"/>
@@ -1327,7 +1339,7 @@
       </c>
       <c r="B60">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C60" t="str">
         <f t="shared" si="1"/>
@@ -1344,7 +1356,7 @@
       </c>
       <c r="B61">
         <f t="shared" si="0"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="1"/>
@@ -1361,7 +1373,7 @@
       </c>
       <c r="B62">
         <f t="shared" si="0"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C62" t="str">
         <f t="shared" si="1"/>
@@ -1378,7 +1390,7 @@
       </c>
       <c r="B63">
         <f t="shared" si="0"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C63" t="str">
         <f t="shared" si="1"/>
@@ -1395,7 +1407,7 @@
       </c>
       <c r="B64">
         <f t="shared" si="0"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C64" t="str">
         <f t="shared" si="1"/>
@@ -1412,7 +1424,7 @@
       </c>
       <c r="B65">
         <f t="shared" si="0"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C65" t="str">
         <f t="shared" si="1"/>
@@ -1429,7 +1441,7 @@
       </c>
       <c r="B66">
         <f t="shared" si="0"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C66" t="str">
         <f t="shared" si="1"/>
@@ -1446,7 +1458,7 @@
       </c>
       <c r="B67">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C67" t="str">
         <f t="shared" si="1"/>
@@ -1496,11 +1508,11 @@
         <v>66</v>
       </c>
       <c r="B70">
-        <f t="shared" ref="B70:B133" si="3">MOD(A70,64)</f>
+        <f t="shared" ref="B70:B133" si="3">MOD(A70,32)</f>
         <v>2</v>
       </c>
       <c r="C70" t="str">
-        <f t="shared" ref="C70:C133" si="4">IF(B70=16, "Failsafe",IF(OR(B70=0,B70=32),"telemetry",""))</f>
+        <f t="shared" ref="C70:C133" si="4">IF(B70=16, "Failsafe",IF(B70=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D70">
@@ -2007,7 +2019,7 @@
       </c>
       <c r="B100">
         <f t="shared" si="3"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C100" t="str">
         <f t="shared" si="4"/>
@@ -2024,7 +2036,7 @@
       </c>
       <c r="B101">
         <f t="shared" si="3"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C101" t="str">
         <f t="shared" si="4"/>
@@ -2041,7 +2053,7 @@
       </c>
       <c r="B102">
         <f t="shared" si="3"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="4"/>
@@ -2058,7 +2070,7 @@
       </c>
       <c r="B103">
         <f t="shared" si="3"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C103" t="str">
         <f t="shared" si="4"/>
@@ -2075,7 +2087,7 @@
       </c>
       <c r="B104">
         <f t="shared" si="3"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C104" t="str">
         <f t="shared" si="4"/>
@@ -2092,7 +2104,7 @@
       </c>
       <c r="B105">
         <f t="shared" si="3"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C105" t="str">
         <f t="shared" si="4"/>
@@ -2109,7 +2121,7 @@
       </c>
       <c r="B106">
         <f t="shared" si="3"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C106" t="str">
         <f t="shared" si="4"/>
@@ -2126,7 +2138,7 @@
       </c>
       <c r="B107">
         <f t="shared" si="3"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C107" t="str">
         <f t="shared" si="4"/>
@@ -2143,7 +2155,7 @@
       </c>
       <c r="B108">
         <f t="shared" si="3"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C108" t="str">
         <f t="shared" si="4"/>
@@ -2160,7 +2172,7 @@
       </c>
       <c r="B109">
         <f t="shared" si="3"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C109" t="str">
         <f t="shared" si="4"/>
@@ -2177,7 +2189,7 @@
       </c>
       <c r="B110">
         <f t="shared" si="3"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="4"/>
@@ -2194,7 +2206,7 @@
       </c>
       <c r="B111">
         <f t="shared" si="3"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C111" t="str">
         <f t="shared" si="4"/>
@@ -2211,7 +2223,7 @@
       </c>
       <c r="B112">
         <f t="shared" si="3"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C112" t="str">
         <f t="shared" si="4"/>
@@ -2228,7 +2240,7 @@
       </c>
       <c r="B113">
         <f t="shared" si="3"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C113" t="str">
         <f t="shared" si="4"/>
@@ -2245,7 +2257,7 @@
       </c>
       <c r="B114">
         <f t="shared" si="3"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C114" t="str">
         <f t="shared" si="4"/>
@@ -2262,7 +2274,7 @@
       </c>
       <c r="B115">
         <f t="shared" si="3"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C115" t="str">
         <f t="shared" si="4"/>
@@ -2279,11 +2291,11 @@
       </c>
       <c r="B116">
         <f t="shared" si="3"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C116" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D116">
         <f t="shared" si="5"/>
@@ -2296,7 +2308,7 @@
       </c>
       <c r="B117">
         <f t="shared" si="3"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C117" t="str">
         <f t="shared" si="4"/>
@@ -2313,7 +2325,7 @@
       </c>
       <c r="B118">
         <f t="shared" si="3"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="4"/>
@@ -2330,7 +2342,7 @@
       </c>
       <c r="B119">
         <f t="shared" si="3"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C119" t="str">
         <f t="shared" si="4"/>
@@ -2347,7 +2359,7 @@
       </c>
       <c r="B120">
         <f t="shared" si="3"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C120" t="str">
         <f t="shared" si="4"/>
@@ -2364,7 +2376,7 @@
       </c>
       <c r="B121">
         <f t="shared" si="3"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C121" t="str">
         <f t="shared" si="4"/>
@@ -2381,7 +2393,7 @@
       </c>
       <c r="B122">
         <f t="shared" si="3"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C122" t="str">
         <f t="shared" si="4"/>
@@ -2398,7 +2410,7 @@
       </c>
       <c r="B123">
         <f t="shared" si="3"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C123" t="str">
         <f t="shared" si="4"/>
@@ -2415,7 +2427,7 @@
       </c>
       <c r="B124">
         <f t="shared" si="3"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C124" t="str">
         <f t="shared" si="4"/>
@@ -2432,7 +2444,7 @@
       </c>
       <c r="B125">
         <f t="shared" si="3"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C125" t="str">
         <f t="shared" si="4"/>
@@ -2449,7 +2461,7 @@
       </c>
       <c r="B126">
         <f t="shared" si="3"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C126" t="str">
         <f t="shared" si="4"/>
@@ -2466,7 +2478,7 @@
       </c>
       <c r="B127">
         <f t="shared" si="3"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C127" t="str">
         <f t="shared" si="4"/>
@@ -2483,7 +2495,7 @@
       </c>
       <c r="B128">
         <f t="shared" si="3"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C128" t="str">
         <f t="shared" si="4"/>
@@ -2500,7 +2512,7 @@
       </c>
       <c r="B129">
         <f t="shared" si="3"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C129" t="str">
         <f t="shared" si="4"/>
@@ -2517,7 +2529,7 @@
       </c>
       <c r="B130">
         <f t="shared" si="3"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C130" t="str">
         <f t="shared" si="4"/>
@@ -2534,7 +2546,7 @@
       </c>
       <c r="B131">
         <f t="shared" si="3"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C131" t="str">
         <f t="shared" si="4"/>
@@ -2584,11 +2596,11 @@
         <v>130</v>
       </c>
       <c r="B134">
-        <f t="shared" ref="B134:B197" si="6">MOD(A134,64)</f>
+        <f t="shared" ref="B134:B197" si="6">MOD(A134,32)</f>
         <v>2</v>
       </c>
       <c r="C134" t="str">
-        <f t="shared" ref="C134:C197" si="7">IF(B134=16, "Failsafe",IF(OR(B134=0,B134=32),"telemetry",""))</f>
+        <f t="shared" ref="C134:C197" si="7">IF(B134=16, "Failsafe",IF(B134=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D134">
@@ -3095,7 +3107,7 @@
       </c>
       <c r="B164">
         <f t="shared" si="6"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C164" t="str">
         <f t="shared" si="7"/>
@@ -3112,7 +3124,7 @@
       </c>
       <c r="B165">
         <f t="shared" si="6"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C165" t="str">
         <f t="shared" si="7"/>
@@ -3129,7 +3141,7 @@
       </c>
       <c r="B166">
         <f t="shared" si="6"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C166" t="str">
         <f t="shared" si="7"/>
@@ -3146,7 +3158,7 @@
       </c>
       <c r="B167">
         <f t="shared" si="6"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C167" t="str">
         <f t="shared" si="7"/>
@@ -3163,7 +3175,7 @@
       </c>
       <c r="B168">
         <f t="shared" si="6"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C168" t="str">
         <f t="shared" si="7"/>
@@ -3180,7 +3192,7 @@
       </c>
       <c r="B169">
         <f t="shared" si="6"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C169" t="str">
         <f t="shared" si="7"/>
@@ -3197,7 +3209,7 @@
       </c>
       <c r="B170">
         <f t="shared" si="6"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C170" t="str">
         <f t="shared" si="7"/>
@@ -3214,7 +3226,7 @@
       </c>
       <c r="B171">
         <f t="shared" si="6"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C171" t="str">
         <f t="shared" si="7"/>
@@ -3231,7 +3243,7 @@
       </c>
       <c r="B172">
         <f t="shared" si="6"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C172" t="str">
         <f t="shared" si="7"/>
@@ -3248,7 +3260,7 @@
       </c>
       <c r="B173">
         <f t="shared" si="6"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C173" t="str">
         <f t="shared" si="7"/>
@@ -3265,7 +3277,7 @@
       </c>
       <c r="B174">
         <f t="shared" si="6"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C174" t="str">
         <f t="shared" si="7"/>
@@ -3282,7 +3294,7 @@
       </c>
       <c r="B175">
         <f t="shared" si="6"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C175" t="str">
         <f t="shared" si="7"/>
@@ -3299,7 +3311,7 @@
       </c>
       <c r="B176">
         <f t="shared" si="6"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C176" t="str">
         <f t="shared" si="7"/>
@@ -3316,7 +3328,7 @@
       </c>
       <c r="B177">
         <f t="shared" si="6"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C177" t="str">
         <f t="shared" si="7"/>
@@ -3333,7 +3345,7 @@
       </c>
       <c r="B178">
         <f t="shared" si="6"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C178" t="str">
         <f t="shared" si="7"/>
@@ -3350,7 +3362,7 @@
       </c>
       <c r="B179">
         <f t="shared" si="6"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C179" t="str">
         <f t="shared" si="7"/>
@@ -3367,11 +3379,11 @@
       </c>
       <c r="B180">
         <f t="shared" si="6"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C180" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D180">
         <f t="shared" si="8"/>
@@ -3384,7 +3396,7 @@
       </c>
       <c r="B181">
         <f t="shared" si="6"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C181" t="str">
         <f t="shared" si="7"/>
@@ -3401,7 +3413,7 @@
       </c>
       <c r="B182">
         <f t="shared" si="6"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C182" t="str">
         <f t="shared" si="7"/>
@@ -3418,7 +3430,7 @@
       </c>
       <c r="B183">
         <f t="shared" si="6"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C183" t="str">
         <f t="shared" si="7"/>
@@ -3435,7 +3447,7 @@
       </c>
       <c r="B184">
         <f t="shared" si="6"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C184" t="str">
         <f t="shared" si="7"/>
@@ -3452,7 +3464,7 @@
       </c>
       <c r="B185">
         <f t="shared" si="6"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C185" t="str">
         <f t="shared" si="7"/>
@@ -3469,7 +3481,7 @@
       </c>
       <c r="B186">
         <f t="shared" si="6"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C186" t="str">
         <f t="shared" si="7"/>
@@ -3486,7 +3498,7 @@
       </c>
       <c r="B187">
         <f t="shared" si="6"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C187" t="str">
         <f t="shared" si="7"/>
@@ -3503,7 +3515,7 @@
       </c>
       <c r="B188">
         <f t="shared" si="6"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C188" t="str">
         <f t="shared" si="7"/>
@@ -3520,7 +3532,7 @@
       </c>
       <c r="B189">
         <f t="shared" si="6"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C189" t="str">
         <f t="shared" si="7"/>
@@ -3537,7 +3549,7 @@
       </c>
       <c r="B190">
         <f t="shared" si="6"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C190" t="str">
         <f t="shared" si="7"/>
@@ -3554,7 +3566,7 @@
       </c>
       <c r="B191">
         <f t="shared" si="6"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C191" t="str">
         <f t="shared" si="7"/>
@@ -3571,7 +3583,7 @@
       </c>
       <c r="B192">
         <f t="shared" si="6"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C192" t="str">
         <f t="shared" si="7"/>
@@ -3588,7 +3600,7 @@
       </c>
       <c r="B193">
         <f t="shared" si="6"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C193" t="str">
         <f t="shared" si="7"/>
@@ -3605,7 +3617,7 @@
       </c>
       <c r="B194">
         <f t="shared" si="6"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C194" t="str">
         <f t="shared" si="7"/>
@@ -3622,7 +3634,7 @@
       </c>
       <c r="B195">
         <f t="shared" si="6"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C195" t="str">
         <f t="shared" si="7"/>
@@ -3672,11 +3684,11 @@
         <v>194</v>
       </c>
       <c r="B198">
-        <f t="shared" ref="B198:B261" si="9">MOD(A198,64)</f>
+        <f t="shared" ref="B198:B261" si="9">MOD(A198,32)</f>
         <v>2</v>
       </c>
       <c r="C198" t="str">
-        <f t="shared" ref="C198:C261" si="10">IF(B198=16, "Failsafe",IF(OR(B198=0,B198=32),"telemetry",""))</f>
+        <f t="shared" ref="C198:C261" si="10">IF(B198=16, "Failsafe",IF(B198=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D198">
@@ -4183,7 +4195,7 @@
       </c>
       <c r="B228">
         <f t="shared" si="9"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C228" t="str">
         <f t="shared" si="10"/>
@@ -4200,7 +4212,7 @@
       </c>
       <c r="B229">
         <f t="shared" si="9"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C229" t="str">
         <f t="shared" si="10"/>
@@ -4217,7 +4229,7 @@
       </c>
       <c r="B230">
         <f t="shared" si="9"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C230" t="str">
         <f t="shared" si="10"/>
@@ -4234,7 +4246,7 @@
       </c>
       <c r="B231">
         <f t="shared" si="9"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C231" t="str">
         <f t="shared" si="10"/>
@@ -4251,7 +4263,7 @@
       </c>
       <c r="B232">
         <f t="shared" si="9"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C232" t="str">
         <f t="shared" si="10"/>
@@ -4268,7 +4280,7 @@
       </c>
       <c r="B233">
         <f t="shared" si="9"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C233" t="str">
         <f t="shared" si="10"/>
@@ -4285,7 +4297,7 @@
       </c>
       <c r="B234">
         <f t="shared" si="9"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C234" t="str">
         <f t="shared" si="10"/>
@@ -4302,7 +4314,7 @@
       </c>
       <c r="B235">
         <f t="shared" si="9"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C235" t="str">
         <f t="shared" si="10"/>
@@ -4319,7 +4331,7 @@
       </c>
       <c r="B236">
         <f t="shared" si="9"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C236" t="str">
         <f t="shared" si="10"/>
@@ -4336,7 +4348,7 @@
       </c>
       <c r="B237">
         <f t="shared" si="9"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C237" t="str">
         <f t="shared" si="10"/>
@@ -4353,7 +4365,7 @@
       </c>
       <c r="B238">
         <f t="shared" si="9"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C238" t="str">
         <f t="shared" si="10"/>
@@ -4370,7 +4382,7 @@
       </c>
       <c r="B239">
         <f t="shared" si="9"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C239" t="str">
         <f t="shared" si="10"/>
@@ -4387,7 +4399,7 @@
       </c>
       <c r="B240">
         <f t="shared" si="9"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C240" t="str">
         <f t="shared" si="10"/>
@@ -4404,7 +4416,7 @@
       </c>
       <c r="B241">
         <f t="shared" si="9"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C241" t="str">
         <f t="shared" si="10"/>
@@ -4421,7 +4433,7 @@
       </c>
       <c r="B242">
         <f t="shared" si="9"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C242" t="str">
         <f t="shared" si="10"/>
@@ -4438,7 +4450,7 @@
       </c>
       <c r="B243">
         <f t="shared" si="9"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C243" t="str">
         <f t="shared" si="10"/>
@@ -4455,11 +4467,11 @@
       </c>
       <c r="B244">
         <f t="shared" si="9"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C244" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D244">
         <f t="shared" si="11"/>
@@ -4472,7 +4484,7 @@
       </c>
       <c r="B245">
         <f t="shared" si="9"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C245" t="str">
         <f t="shared" si="10"/>
@@ -4489,7 +4501,7 @@
       </c>
       <c r="B246">
         <f t="shared" si="9"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C246" t="str">
         <f t="shared" si="10"/>
@@ -4506,7 +4518,7 @@
       </c>
       <c r="B247">
         <f t="shared" si="9"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C247" t="str">
         <f t="shared" si="10"/>
@@ -4523,7 +4535,7 @@
       </c>
       <c r="B248">
         <f t="shared" si="9"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C248" t="str">
         <f t="shared" si="10"/>
@@ -4540,7 +4552,7 @@
       </c>
       <c r="B249">
         <f t="shared" si="9"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C249" t="str">
         <f t="shared" si="10"/>
@@ -4557,7 +4569,7 @@
       </c>
       <c r="B250">
         <f t="shared" si="9"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C250" t="str">
         <f t="shared" si="10"/>
@@ -4574,7 +4586,7 @@
       </c>
       <c r="B251">
         <f t="shared" si="9"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C251" t="str">
         <f t="shared" si="10"/>
@@ -4591,7 +4603,7 @@
       </c>
       <c r="B252">
         <f t="shared" si="9"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C252" t="str">
         <f t="shared" si="10"/>
@@ -4608,7 +4620,7 @@
       </c>
       <c r="B253">
         <f t="shared" si="9"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C253" t="str">
         <f t="shared" si="10"/>
@@ -4625,7 +4637,7 @@
       </c>
       <c r="B254">
         <f t="shared" si="9"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C254" t="str">
         <f t="shared" si="10"/>
@@ -4642,7 +4654,7 @@
       </c>
       <c r="B255">
         <f t="shared" si="9"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C255" t="str">
         <f t="shared" si="10"/>
@@ -4659,7 +4671,7 @@
       </c>
       <c r="B256">
         <f t="shared" si="9"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C256" t="str">
         <f t="shared" si="10"/>
@@ -4676,7 +4688,7 @@
       </c>
       <c r="B257">
         <f t="shared" si="9"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C257" t="str">
         <f t="shared" si="10"/>
@@ -4693,7 +4705,7 @@
       </c>
       <c r="B258">
         <f t="shared" si="9"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C258" t="str">
         <f t="shared" si="10"/>
@@ -4710,7 +4722,7 @@
       </c>
       <c r="B259">
         <f t="shared" si="9"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C259" t="str">
         <f t="shared" si="10"/>
@@ -4760,11 +4772,11 @@
         <v>258</v>
       </c>
       <c r="B262">
-        <f t="shared" ref="B262:B325" si="12">MOD(A262,64)</f>
+        <f t="shared" ref="B262:B325" si="12">MOD(A262,32)</f>
         <v>2</v>
       </c>
       <c r="C262" t="str">
-        <f t="shared" ref="C262:C325" si="13">IF(B262=16, "Failsafe",IF(OR(B262=0,B262=32),"telemetry",""))</f>
+        <f t="shared" ref="C262:C325" si="13">IF(B262=16, "Failsafe",IF(B262=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D262">
@@ -5271,7 +5283,7 @@
       </c>
       <c r="B292">
         <f t="shared" si="12"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C292" t="str">
         <f t="shared" si="13"/>
@@ -5288,7 +5300,7 @@
       </c>
       <c r="B293">
         <f t="shared" si="12"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C293" t="str">
         <f t="shared" si="13"/>
@@ -5305,7 +5317,7 @@
       </c>
       <c r="B294">
         <f t="shared" si="12"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C294" t="str">
         <f t="shared" si="13"/>
@@ -5322,7 +5334,7 @@
       </c>
       <c r="B295">
         <f t="shared" si="12"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C295" t="str">
         <f t="shared" si="13"/>
@@ -5339,7 +5351,7 @@
       </c>
       <c r="B296">
         <f t="shared" si="12"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C296" t="str">
         <f t="shared" si="13"/>
@@ -5356,7 +5368,7 @@
       </c>
       <c r="B297">
         <f t="shared" si="12"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C297" t="str">
         <f t="shared" si="13"/>
@@ -5373,7 +5385,7 @@
       </c>
       <c r="B298">
         <f t="shared" si="12"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C298" t="str">
         <f t="shared" si="13"/>
@@ -5390,7 +5402,7 @@
       </c>
       <c r="B299">
         <f t="shared" si="12"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C299" t="str">
         <f t="shared" si="13"/>
@@ -5407,7 +5419,7 @@
       </c>
       <c r="B300">
         <f t="shared" si="12"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C300" t="str">
         <f t="shared" si="13"/>
@@ -5424,7 +5436,7 @@
       </c>
       <c r="B301">
         <f t="shared" si="12"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C301" t="str">
         <f t="shared" si="13"/>
@@ -5441,7 +5453,7 @@
       </c>
       <c r="B302">
         <f t="shared" si="12"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C302" t="str">
         <f t="shared" si="13"/>
@@ -5458,7 +5470,7 @@
       </c>
       <c r="B303">
         <f t="shared" si="12"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C303" t="str">
         <f t="shared" si="13"/>
@@ -5475,7 +5487,7 @@
       </c>
       <c r="B304">
         <f t="shared" si="12"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C304" t="str">
         <f t="shared" si="13"/>
@@ -5492,7 +5504,7 @@
       </c>
       <c r="B305">
         <f t="shared" si="12"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C305" t="str">
         <f t="shared" si="13"/>
@@ -5509,7 +5521,7 @@
       </c>
       <c r="B306">
         <f t="shared" si="12"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C306" t="str">
         <f t="shared" si="13"/>
@@ -5526,7 +5538,7 @@
       </c>
       <c r="B307">
         <f t="shared" si="12"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C307" t="str">
         <f t="shared" si="13"/>
@@ -5543,11 +5555,11 @@
       </c>
       <c r="B308">
         <f t="shared" si="12"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C308" t="str">
         <f t="shared" si="13"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D308">
         <f t="shared" si="14"/>
@@ -5560,7 +5572,7 @@
       </c>
       <c r="B309">
         <f t="shared" si="12"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C309" t="str">
         <f t="shared" si="13"/>
@@ -5577,7 +5589,7 @@
       </c>
       <c r="B310">
         <f t="shared" si="12"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C310" t="str">
         <f t="shared" si="13"/>
@@ -5594,7 +5606,7 @@
       </c>
       <c r="B311">
         <f t="shared" si="12"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C311" t="str">
         <f t="shared" si="13"/>
@@ -5611,7 +5623,7 @@
       </c>
       <c r="B312">
         <f t="shared" si="12"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C312" t="str">
         <f t="shared" si="13"/>
@@ -5628,7 +5640,7 @@
       </c>
       <c r="B313">
         <f t="shared" si="12"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C313" t="str">
         <f t="shared" si="13"/>
@@ -5645,7 +5657,7 @@
       </c>
       <c r="B314">
         <f t="shared" si="12"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C314" t="str">
         <f t="shared" si="13"/>
@@ -5662,7 +5674,7 @@
       </c>
       <c r="B315">
         <f t="shared" si="12"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C315" t="str">
         <f t="shared" si="13"/>
@@ -5679,7 +5691,7 @@
       </c>
       <c r="B316">
         <f t="shared" si="12"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C316" t="str">
         <f t="shared" si="13"/>
@@ -5696,7 +5708,7 @@
       </c>
       <c r="B317">
         <f t="shared" si="12"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C317" t="str">
         <f t="shared" si="13"/>
@@ -5713,7 +5725,7 @@
       </c>
       <c r="B318">
         <f t="shared" si="12"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C318" t="str">
         <f t="shared" si="13"/>
@@ -5730,7 +5742,7 @@
       </c>
       <c r="B319">
         <f t="shared" si="12"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C319" t="str">
         <f t="shared" si="13"/>
@@ -5747,7 +5759,7 @@
       </c>
       <c r="B320">
         <f t="shared" si="12"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C320" t="str">
         <f t="shared" si="13"/>
@@ -5764,7 +5776,7 @@
       </c>
       <c r="B321">
         <f t="shared" si="12"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C321" t="str">
         <f t="shared" si="13"/>
@@ -5781,7 +5793,7 @@
       </c>
       <c r="B322">
         <f t="shared" si="12"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C322" t="str">
         <f t="shared" si="13"/>
@@ -5798,7 +5810,7 @@
       </c>
       <c r="B323">
         <f t="shared" si="12"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C323" t="str">
         <f t="shared" si="13"/>
@@ -5848,11 +5860,11 @@
         <v>322</v>
       </c>
       <c r="B326">
-        <f t="shared" ref="B326:B389" si="15">MOD(A326,64)</f>
+        <f t="shared" ref="B326:B389" si="15">MOD(A326,32)</f>
         <v>2</v>
       </c>
       <c r="C326" t="str">
-        <f t="shared" ref="C326:C389" si="16">IF(B326=16, "Failsafe",IF(OR(B326=0,B326=32),"telemetry",""))</f>
+        <f t="shared" ref="C326:C389" si="16">IF(B326=16, "Failsafe",IF(B326=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D326">
@@ -6359,7 +6371,7 @@
       </c>
       <c r="B356">
         <f t="shared" si="15"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C356" t="str">
         <f t="shared" si="16"/>
@@ -6376,7 +6388,7 @@
       </c>
       <c r="B357">
         <f t="shared" si="15"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C357" t="str">
         <f t="shared" si="16"/>
@@ -6393,7 +6405,7 @@
       </c>
       <c r="B358">
         <f t="shared" si="15"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C358" t="str">
         <f t="shared" si="16"/>
@@ -6410,7 +6422,7 @@
       </c>
       <c r="B359">
         <f t="shared" si="15"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C359" t="str">
         <f t="shared" si="16"/>
@@ -6427,7 +6439,7 @@
       </c>
       <c r="B360">
         <f t="shared" si="15"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C360" t="str">
         <f t="shared" si="16"/>
@@ -6444,7 +6456,7 @@
       </c>
       <c r="B361">
         <f t="shared" si="15"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C361" t="str">
         <f t="shared" si="16"/>
@@ -6461,7 +6473,7 @@
       </c>
       <c r="B362">
         <f t="shared" si="15"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C362" t="str">
         <f t="shared" si="16"/>
@@ -6478,7 +6490,7 @@
       </c>
       <c r="B363">
         <f t="shared" si="15"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C363" t="str">
         <f t="shared" si="16"/>
@@ -6495,7 +6507,7 @@
       </c>
       <c r="B364">
         <f t="shared" si="15"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C364" t="str">
         <f t="shared" si="16"/>
@@ -6512,7 +6524,7 @@
       </c>
       <c r="B365">
         <f t="shared" si="15"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C365" t="str">
         <f t="shared" si="16"/>
@@ -6529,7 +6541,7 @@
       </c>
       <c r="B366">
         <f t="shared" si="15"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C366" t="str">
         <f t="shared" si="16"/>
@@ -6546,7 +6558,7 @@
       </c>
       <c r="B367">
         <f t="shared" si="15"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C367" t="str">
         <f t="shared" si="16"/>
@@ -6563,7 +6575,7 @@
       </c>
       <c r="B368">
         <f t="shared" si="15"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C368" t="str">
         <f t="shared" si="16"/>
@@ -6580,7 +6592,7 @@
       </c>
       <c r="B369">
         <f t="shared" si="15"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C369" t="str">
         <f t="shared" si="16"/>
@@ -6597,7 +6609,7 @@
       </c>
       <c r="B370">
         <f t="shared" si="15"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C370" t="str">
         <f t="shared" si="16"/>
@@ -6614,7 +6626,7 @@
       </c>
       <c r="B371">
         <f t="shared" si="15"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C371" t="str">
         <f t="shared" si="16"/>
@@ -6631,11 +6643,11 @@
       </c>
       <c r="B372">
         <f t="shared" si="15"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C372" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D372">
         <f t="shared" si="17"/>
@@ -6648,7 +6660,7 @@
       </c>
       <c r="B373">
         <f t="shared" si="15"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C373" t="str">
         <f t="shared" si="16"/>
@@ -6665,7 +6677,7 @@
       </c>
       <c r="B374">
         <f t="shared" si="15"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C374" t="str">
         <f t="shared" si="16"/>
@@ -6682,7 +6694,7 @@
       </c>
       <c r="B375">
         <f t="shared" si="15"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C375" t="str">
         <f t="shared" si="16"/>
@@ -6699,7 +6711,7 @@
       </c>
       <c r="B376">
         <f t="shared" si="15"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C376" t="str">
         <f t="shared" si="16"/>
@@ -6716,7 +6728,7 @@
       </c>
       <c r="B377">
         <f t="shared" si="15"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C377" t="str">
         <f t="shared" si="16"/>
@@ -6733,7 +6745,7 @@
       </c>
       <c r="B378">
         <f t="shared" si="15"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C378" t="str">
         <f t="shared" si="16"/>
@@ -6750,7 +6762,7 @@
       </c>
       <c r="B379">
         <f t="shared" si="15"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C379" t="str">
         <f t="shared" si="16"/>
@@ -6767,7 +6779,7 @@
       </c>
       <c r="B380">
         <f t="shared" si="15"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C380" t="str">
         <f t="shared" si="16"/>
@@ -6784,7 +6796,7 @@
       </c>
       <c r="B381">
         <f t="shared" si="15"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C381" t="str">
         <f t="shared" si="16"/>
@@ -6801,7 +6813,7 @@
       </c>
       <c r="B382">
         <f t="shared" si="15"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C382" t="str">
         <f t="shared" si="16"/>
@@ -6818,7 +6830,7 @@
       </c>
       <c r="B383">
         <f t="shared" si="15"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C383" t="str">
         <f t="shared" si="16"/>
@@ -6835,7 +6847,7 @@
       </c>
       <c r="B384">
         <f t="shared" si="15"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C384" t="str">
         <f t="shared" si="16"/>
@@ -6852,7 +6864,7 @@
       </c>
       <c r="B385">
         <f t="shared" si="15"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C385" t="str">
         <f t="shared" si="16"/>
@@ -6869,7 +6881,7 @@
       </c>
       <c r="B386">
         <f t="shared" si="15"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C386" t="str">
         <f t="shared" si="16"/>
@@ -6886,7 +6898,7 @@
       </c>
       <c r="B387">
         <f t="shared" si="15"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C387" t="str">
         <f t="shared" si="16"/>
@@ -6936,11 +6948,11 @@
         <v>386</v>
       </c>
       <c r="B390">
-        <f t="shared" ref="B390:B453" si="18">MOD(A390,64)</f>
+        <f t="shared" ref="B390:B453" si="18">MOD(A390,32)</f>
         <v>2</v>
       </c>
       <c r="C390" t="str">
-        <f t="shared" ref="C390:C453" si="19">IF(B390=16, "Failsafe",IF(OR(B390=0,B390=32),"telemetry",""))</f>
+        <f t="shared" ref="C390:C453" si="19">IF(B390=16, "Failsafe",IF(B390=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D390">
@@ -7447,7 +7459,7 @@
       </c>
       <c r="B420">
         <f t="shared" si="18"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C420" t="str">
         <f t="shared" si="19"/>
@@ -7464,7 +7476,7 @@
       </c>
       <c r="B421">
         <f t="shared" si="18"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C421" t="str">
         <f t="shared" si="19"/>
@@ -7481,7 +7493,7 @@
       </c>
       <c r="B422">
         <f t="shared" si="18"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C422" t="str">
         <f t="shared" si="19"/>
@@ -7498,7 +7510,7 @@
       </c>
       <c r="B423">
         <f t="shared" si="18"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C423" t="str">
         <f t="shared" si="19"/>
@@ -7515,7 +7527,7 @@
       </c>
       <c r="B424">
         <f t="shared" si="18"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C424" t="str">
         <f t="shared" si="19"/>
@@ -7532,7 +7544,7 @@
       </c>
       <c r="B425">
         <f t="shared" si="18"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C425" t="str">
         <f t="shared" si="19"/>
@@ -7549,7 +7561,7 @@
       </c>
       <c r="B426">
         <f t="shared" si="18"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C426" t="str">
         <f t="shared" si="19"/>
@@ -7566,7 +7578,7 @@
       </c>
       <c r="B427">
         <f t="shared" si="18"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C427" t="str">
         <f t="shared" si="19"/>
@@ -7583,7 +7595,7 @@
       </c>
       <c r="B428">
         <f t="shared" si="18"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C428" t="str">
         <f t="shared" si="19"/>
@@ -7600,7 +7612,7 @@
       </c>
       <c r="B429">
         <f t="shared" si="18"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C429" t="str">
         <f t="shared" si="19"/>
@@ -7617,7 +7629,7 @@
       </c>
       <c r="B430">
         <f t="shared" si="18"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C430" t="str">
         <f t="shared" si="19"/>
@@ -7634,7 +7646,7 @@
       </c>
       <c r="B431">
         <f t="shared" si="18"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C431" t="str">
         <f t="shared" si="19"/>
@@ -7651,7 +7663,7 @@
       </c>
       <c r="B432">
         <f t="shared" si="18"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C432" t="str">
         <f t="shared" si="19"/>
@@ -7668,7 +7680,7 @@
       </c>
       <c r="B433">
         <f t="shared" si="18"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C433" t="str">
         <f t="shared" si="19"/>
@@ -7685,7 +7697,7 @@
       </c>
       <c r="B434">
         <f t="shared" si="18"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C434" t="str">
         <f t="shared" si="19"/>
@@ -7702,7 +7714,7 @@
       </c>
       <c r="B435">
         <f t="shared" si="18"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C435" t="str">
         <f t="shared" si="19"/>
@@ -7719,11 +7731,11 @@
       </c>
       <c r="B436">
         <f t="shared" si="18"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C436" t="str">
         <f t="shared" si="19"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D436">
         <f t="shared" si="20"/>
@@ -7736,7 +7748,7 @@
       </c>
       <c r="B437">
         <f t="shared" si="18"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C437" t="str">
         <f t="shared" si="19"/>
@@ -7753,7 +7765,7 @@
       </c>
       <c r="B438">
         <f t="shared" si="18"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C438" t="str">
         <f t="shared" si="19"/>
@@ -7770,7 +7782,7 @@
       </c>
       <c r="B439">
         <f t="shared" si="18"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C439" t="str">
         <f t="shared" si="19"/>
@@ -7787,7 +7799,7 @@
       </c>
       <c r="B440">
         <f t="shared" si="18"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C440" t="str">
         <f t="shared" si="19"/>
@@ -7804,7 +7816,7 @@
       </c>
       <c r="B441">
         <f t="shared" si="18"/>
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C441" t="str">
         <f t="shared" si="19"/>
@@ -7821,7 +7833,7 @@
       </c>
       <c r="B442">
         <f t="shared" si="18"/>
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="C442" t="str">
         <f t="shared" si="19"/>
@@ -7838,7 +7850,7 @@
       </c>
       <c r="B443">
         <f t="shared" si="18"/>
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="C443" t="str">
         <f t="shared" si="19"/>
@@ -7855,7 +7867,7 @@
       </c>
       <c r="B444">
         <f t="shared" si="18"/>
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="C444" t="str">
         <f t="shared" si="19"/>
@@ -7872,7 +7884,7 @@
       </c>
       <c r="B445">
         <f t="shared" si="18"/>
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="C445" t="str">
         <f t="shared" si="19"/>
@@ -7889,7 +7901,7 @@
       </c>
       <c r="B446">
         <f t="shared" si="18"/>
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="C446" t="str">
         <f t="shared" si="19"/>
@@ -7906,7 +7918,7 @@
       </c>
       <c r="B447">
         <f t="shared" si="18"/>
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C447" t="str">
         <f t="shared" si="19"/>
@@ -7923,7 +7935,7 @@
       </c>
       <c r="B448">
         <f t="shared" si="18"/>
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="C448" t="str">
         <f t="shared" si="19"/>
@@ -7940,7 +7952,7 @@
       </c>
       <c r="B449">
         <f t="shared" si="18"/>
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C449" t="str">
         <f t="shared" si="19"/>
@@ -7957,7 +7969,7 @@
       </c>
       <c r="B450">
         <f t="shared" si="18"/>
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C450" t="str">
         <f t="shared" si="19"/>
@@ -7974,7 +7986,7 @@
       </c>
       <c r="B451">
         <f t="shared" si="18"/>
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C451" t="str">
         <f t="shared" si="19"/>
@@ -8024,11 +8036,11 @@
         <v>450</v>
       </c>
       <c r="B454">
-        <f t="shared" ref="B454:B504" si="21">MOD(A454,64)</f>
+        <f t="shared" ref="B454:B504" si="21">MOD(A454,32)</f>
         <v>2</v>
       </c>
       <c r="C454" t="str">
-        <f t="shared" ref="C454:C504" si="22">IF(B454=16, "Failsafe",IF(OR(B454=0,B454=32),"telemetry",""))</f>
+        <f t="shared" ref="C454:C504" si="22">IF(B454=16, "Failsafe",IF(B454=0,"telemetry",""))</f>
         <v/>
       </c>
       <c r="D454">
@@ -8535,7 +8547,7 @@
       </c>
       <c r="B484">
         <f t="shared" si="21"/>
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="C484" t="str">
         <f t="shared" si="22"/>
@@ -8552,7 +8564,7 @@
       </c>
       <c r="B485">
         <f t="shared" si="21"/>
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="C485" t="str">
         <f t="shared" si="22"/>
@@ -8569,7 +8581,7 @@
       </c>
       <c r="B486">
         <f t="shared" si="21"/>
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="C486" t="str">
         <f t="shared" si="22"/>
@@ -8586,7 +8598,7 @@
       </c>
       <c r="B487">
         <f t="shared" si="21"/>
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C487" t="str">
         <f t="shared" si="22"/>
@@ -8603,7 +8615,7 @@
       </c>
       <c r="B488">
         <f t="shared" si="21"/>
-        <v>36</v>
+        <v>4</v>
       </c>
       <c r="C488" t="str">
         <f t="shared" si="22"/>
@@ -8620,7 +8632,7 @@
       </c>
       <c r="B489">
         <f t="shared" si="21"/>
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C489" t="str">
         <f t="shared" si="22"/>
@@ -8637,7 +8649,7 @@
       </c>
       <c r="B490">
         <f t="shared" si="21"/>
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="C490" t="str">
         <f t="shared" si="22"/>
@@ -8654,7 +8666,7 @@
       </c>
       <c r="B491">
         <f t="shared" si="21"/>
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="C491" t="str">
         <f t="shared" si="22"/>
@@ -8671,7 +8683,7 @@
       </c>
       <c r="B492">
         <f t="shared" si="21"/>
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C492" t="str">
         <f t="shared" si="22"/>
@@ -8688,7 +8700,7 @@
       </c>
       <c r="B493">
         <f t="shared" si="21"/>
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C493" t="str">
         <f t="shared" si="22"/>
@@ -8705,7 +8717,7 @@
       </c>
       <c r="B494">
         <f t="shared" si="21"/>
-        <v>42</v>
+        <v>10</v>
       </c>
       <c r="C494" t="str">
         <f t="shared" si="22"/>
@@ -8722,7 +8734,7 @@
       </c>
       <c r="B495">
         <f t="shared" si="21"/>
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="C495" t="str">
         <f t="shared" si="22"/>
@@ -8739,7 +8751,7 @@
       </c>
       <c r="B496">
         <f t="shared" si="21"/>
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C496" t="str">
         <f t="shared" si="22"/>
@@ -8756,7 +8768,7 @@
       </c>
       <c r="B497">
         <f t="shared" si="21"/>
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C497" t="str">
         <f t="shared" si="22"/>
@@ -8773,7 +8785,7 @@
       </c>
       <c r="B498">
         <f t="shared" si="21"/>
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="C498" t="str">
         <f t="shared" si="22"/>
@@ -8790,7 +8802,7 @@
       </c>
       <c r="B499">
         <f t="shared" si="21"/>
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="C499" t="str">
         <f t="shared" si="22"/>
@@ -8807,11 +8819,11 @@
       </c>
       <c r="B500">
         <f t="shared" si="21"/>
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="C500" t="str">
         <f t="shared" si="22"/>
-        <v/>
+        <v>Failsafe</v>
       </c>
       <c r="D500">
         <f t="shared" si="23"/>
@@ -8824,7 +8836,7 @@
       </c>
       <c r="B501">
         <f t="shared" si="21"/>
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C501" t="str">
         <f t="shared" si="22"/>
@@ -8841,7 +8853,7 @@
       </c>
       <c r="B502">
         <f t="shared" si="21"/>
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C502" t="str">
         <f t="shared" si="22"/>
@@ -8858,7 +8870,7 @@
       </c>
       <c r="B503">
         <f t="shared" si="21"/>
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="C503" t="str">
         <f t="shared" si="22"/>
@@ -8875,7 +8887,7 @@
       </c>
       <c r="B504">
         <f t="shared" si="21"/>
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="C504" t="str">
         <f t="shared" si="22"/>

</xml_diff>